<commit_message>
Affärskort i personkortsleken och fler vägar till personkort
- Personkort: budstrid, övertagande, gratis uppgradering, omförhandlat lån, DD-val och
  konvertering ersätter 3 förhandlings- och 3 energikort (73 → 81).
- Omvärld: personkort per hyresrätt/kontor, mentorsprogram, köparnas marknad (31 → 35).
- Kvartal: personkort per fastighet av fokustypen i varje typlek (46 → 50).
- Motorn hanterar effekterna; bottarna värderar tvångsbud i F-värde.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_kvartalskort.xlsx
+++ b/kortdata/F_kvartalskort.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2064,6 +2064,142 @@
         </is>
       </c>
       <c r="H47" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>QHR-11</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>HYRESRÄTT</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>personkort_fokus</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Hyresgästföreningen bjuder in</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Dialogen om hyrorna öppnar dörrar. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>QFO-13</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>FÖRSKOLA</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>personkort_fokus</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Kommunen söker samarbetspartner</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Förskoleförvaltningen vill teckna långa avtal. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>QLO-13</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>LOKAL</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>personkort_fokus</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Handelsdagarna</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Butikskedjorna letar nya lägen. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>QKO-13</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>KONTOR</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>personkort_fokus</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Företagen flyttar ihop</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Hybridarbetet ger nya behov av kontor. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2114,7 +2250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2824,6 +2960,66 @@
         </is>
       </c>
       <c r="C47" t="inlineStr">
+        <is>
+          <t>ej bestämt</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Hyresgästföreningen bjuder in</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ej bestämt</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Kommunen söker samarbetspartner</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ej bestämt</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Handelsdagarna</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ej bestämt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Företagen flyttar ihop</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
         <is>
           <t>ej bestämt</t>
         </is>
@@ -3097,7 +3293,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>46 (kortspecen: 46)</t>
+          <t>50 (kortspecen: 50)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Förvaltningens handlek byter namn: personkort → nätverkskort
Undviker krock med personkort (CEO/CFO/COO) och personalkort (PC/AC/FC/FS). Gäller bara
otryckta kort: F-CSV:er, F_nätverkskort.xlsx, effektkoder (dra_natverkskort m.fl.), motorn,
specen, designdokumentet och regelbokens kapitel 9.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_kvartalskort.xlsx
+++ b/kortdata/F_kvartalskort.xlsx
@@ -2083,7 +2083,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>personkort_fokus</t>
+          <t>natverkskort_fokus</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Dialogen om hyrorna öppnar dörrar. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+          <t>Dialogen om hyrorna öppnar dörrar. Varje spelare drar ett nätverkskort per egen fastighet av typen.</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>personkort_fokus</t>
+          <t>natverkskort_fokus</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Förskoleförvaltningen vill teckna långa avtal. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+          <t>Förskoleförvaltningen vill teckna långa avtal. Varje spelare drar ett nätverkskort per egen fastighet av typen.</t>
         </is>
       </c>
       <c r="H49" s="2" t="n">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>personkort_fokus</t>
+          <t>natverkskort_fokus</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Butikskedjorna letar nya lägen. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+          <t>Butikskedjorna letar nya lägen. Varje spelare drar ett nätverkskort per egen fastighet av typen.</t>
         </is>
       </c>
       <c r="H50" s="2" t="n">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>personkort_fokus</t>
+          <t>natverkskort_fokus</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Hybridarbetet ger nya behov av kontor. Varje spelare drar ett personkort per egen fastighet av typen.</t>
+          <t>Hybridarbetet ger nya behov av kontor. Varje spelare drar ett nätverkskort per egen fastighet av typen.</t>
         </is>
       </c>
       <c r="H51" s="2" t="n">

</xml_diff>